<commit_message>
Create JOb api data driven test
</commit_message>
<xml_diff>
--- a/src/test/resources/test-data/LoginCreds.xlsx
+++ b/src/test/resources/test-data/LoginCreds.xlsx
@@ -1,40 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68672ACF-CFBA-4751-94E1-E5CC3DCB9407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" name="LoginTestData" sheetId="1"/>
+    <sheet r:id="rId2" name="CreateJobTestData" sheetId="2"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>username</t>
   </si>
@@ -52,18 +54,142 @@
   </si>
   <si>
     <t>iamqc</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Sachin</t>
+  </si>
+  <si>
+    <t>Lad</t>
+  </si>
+  <si>
+    <t>sonawaneom617@gmail.com</t>
+  </si>
+  <si>
+    <t>AG</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>PG</t>
+  </si>
+  <si>
+    <t>pune</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>2025-09-23T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>11683097935667</t>
+  </si>
+  <si>
+    <t>gyu</t>
+  </si>
+  <si>
+    <t>12683097935667</t>
+  </si>
+  <si>
+    <t>13683097935667</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -84,26 +210,43 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -149,7 +292,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -201,7 +344,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -262,171 +405,175 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{399CDA92-BCEE-481D-A0D9-2B74F3DDBFEE}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,7 +581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -442,7 +589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -450,7 +597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -458,7 +605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -467,6 +614,389 @@
       </c>
     </row>
   </sheetData>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5C970423-3E01-483E-81AE-682547B15393}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:AA4"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.28125" customWidth="1"/>
+    <col min="3" max="3" width="21.8515625" customWidth="1"/>
+    <col min="4" max="4" width="11.57421875" customWidth="1"/>
+    <col min="5" max="5" width="20.421875" customWidth="1"/>
+    <col min="6" max="6" width="20.28125" customWidth="1"/>
+    <col min="7" max="7" width="25.00390625" customWidth="1"/>
+    <col min="8" max="8" style="1" width="28.28125" customWidth="1"/>
+    <col min="9" max="10" width="27.28125" customWidth="1"/>
+    <col min="11" max="11" width="29.8515625" customWidth="1"/>
+    <col min="12" max="12" width="34.421875" customWidth="1"/>
+    <col min="13" max="13" width="30.28125" customWidth="1"/>
+    <col min="14" max="14" width="27.57421875" customWidth="1"/>
+    <col min="15" max="15" width="23.00390625" customWidth="1"/>
+    <col min="16" max="16" width="26.28125" customWidth="1"/>
+    <col min="17" max="17" width="25.8515625" customWidth="1"/>
+    <col min="18" max="18" width="23.57421875" customWidth="1"/>
+    <col min="19" max="19" width="25.00390625" customWidth="1"/>
+    <col min="20" max="20" width="31.7109375" customWidth="1"/>
+    <col min="21" max="22" width="23.8515625" customWidth="1"/>
+    <col min="23" max="23" width="25.00390625" customWidth="1"/>
+    <col min="24" max="24" width="28.421875" customWidth="1"/>
+    <col min="25" max="25" width="31.421875" customWidth="1"/>
+    <col min="26" max="26" width="12.7109375" customWidth="1"/>
+    <col min="27" max="27" width="17.421875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" t="s">
+        <v>26</v>
+      </c>
+      <c r="V1" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" t="s">
+        <v>28</v>
+      </c>
+      <c r="X1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2">
+        <v>8474563674</v>
+      </c>
+      <c r="H2" s="1">
+        <v>8474563674</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2">
+        <v>411052</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="W2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X2">
+        <v>3</v>
+      </c>
+      <c r="Y2">
+        <v>3</v>
+      </c>
+      <c r="Z2">
+        <v>6</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3">
+        <v>8474563674</v>
+      </c>
+      <c r="H3" s="1">
+        <v>8474563674</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3">
+        <v>411052</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" t="s">
+        <v>42</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="W3" t="s">
+        <v>42</v>
+      </c>
+      <c r="X3">
+        <v>3</v>
+      </c>
+      <c r="Y3">
+        <v>3</v>
+      </c>
+      <c r="Z3">
+        <v>6</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4">
+        <v>8474563674</v>
+      </c>
+      <c r="H4" s="1">
+        <v>8474563674</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4">
+        <v>411052</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" t="s">
+        <v>42</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="W4" t="s">
+        <v>42</v>
+      </c>
+      <c r="X4">
+        <v>3</v>
+      </c>
+      <c r="Y4">
+        <v>3</v>
+      </c>
+      <c r="Z4">
+        <v>6</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>